<commit_message>
v2.1: Dual Linter and UI — Vacuum engine, interactive filters, ImportDialog extraction, tab coloring, body examples (builds 2.1.28-2.1.42)
</commit_message>
<xml_diff>
--- a/Templates Converted/amendChangeSettlementBIC.230511.xlsx
+++ b/Templates Converted/amendChangeSettlementBIC.230511.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="Questa_cartella_di_lavoro"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
@@ -210,6 +210,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -217,9 +220,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -609,19 +609,19 @@
           <t>Request Parameters</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="14" t="n"/>
-      <c r="J1" s="14" t="n"/>
-      <c r="K1" s="14" t="n"/>
-      <c r="L1" s="14" t="n"/>
-      <c r="M1" s="14" t="n"/>
-      <c r="N1" s="14" t="n"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
+      <c r="G1" s="15" t="n"/>
+      <c r="H1" s="15" t="n"/>
+      <c r="I1" s="15" t="n"/>
+      <c r="J1" s="15" t="n"/>
+      <c r="K1" s="15" t="n"/>
+      <c r="L1" s="15" t="n"/>
+      <c r="M1" s="15" t="n"/>
+      <c r="N1" s="15" t="n"/>
     </row>
     <row r="2" ht="57.6" customFormat="1" customHeight="1" s="4">
       <c r="A2" s="1" t="inlineStr">
@@ -629,7 +629,7 @@
           <t>Name</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -704,7 +704,7 @@
           <t>senderBIC</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>The BIC sending the request
 **ValidationRule(s)** It must be equal to the BIC of the DP certificate (errorCode XA02)
@@ -753,15 +753,15 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFFF9999"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
     <col width="19" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
     <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
@@ -889,43 +889,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>ErrorResponse</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -935,15 +898,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFFF9999"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
     <col width="23" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
     <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
@@ -1071,43 +1034,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>ErrorResponse</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -1121,13 +1047,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="14" customWidth="1" style="3" min="1" max="1"/>
-    <col width="49" customWidth="1" style="3" min="2" max="4"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" style="3" min="2" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
     <col width="18" customWidth="1" style="3" min="6" max="6"/>
     <col width="42" customWidth="1" style="3" min="7" max="7"/>
@@ -1139,7 +1065,6 @@
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="63" customHeight="1">
@@ -1148,17 +1073,9 @@
           <t>Request Body</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Structure of a FPAD account assessment request.</t>
-        </is>
-      </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="n"/>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
       <c r="E1" s="8" t="n"/>
       <c r="F1" s="8" t="n"/>
       <c r="G1" s="8" t="n"/>
@@ -1170,7 +1087,6 @@
       <c r="M1" s="8" t="n"/>
       <c r="N1" s="8" t="n"/>
       <c r="O1" s="8" t="n"/>
-      <c r="P1" s="12" t="n"/>
     </row>
     <row r="2" ht="43.15" customFormat="1" customHeight="1" s="4">
       <c r="A2" s="1" t="inlineStr">
@@ -1188,7 +1104,7 @@
           <t>Parent</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -1252,7 +1168,6 @@
           <t>Example</t>
         </is>
       </c>
-      <c r="P2" s="12" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -1266,7 +1181,7 @@
         </is>
       </c>
       <c r="C3" s="12" t="n"/>
-      <c r="D3" s="16" t="n"/>
+      <c r="D3" s="12" t="n"/>
       <c r="E3" s="12" t="inlineStr">
         <is>
           <t>schema</t>
@@ -1290,616 +1205,6 @@
       <c r="M3" s="12" t="n"/>
       <c r="N3" s="12" t="n"/>
       <c r="O3" s="12" t="n"/>
-      <c r="P3" s="12" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>dateTime</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>The date and time of the API Request creation</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n"/>
-      <c r="K4" s="12" t="n"/>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>settlementBIC</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n"/>
-      <c r="K5" s="12" t="n"/>
-      <c r="L5" s="12" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="12" t="n"/>
-      <c r="O5" s="12" t="n"/>
-      <c r="P5" s="12" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICCode</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>settlementBIC</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>The Settlement BIC adhering to CGS. This is the settlement BIC of the STEP2 DP Preferred Agent in the relevant Step2 service.
-**ValidationRule(s)** It must correspond to the Settlement BIC of the Preferred Agent sending the request
-(errorCode PY01)
-It must be present in the system and it must not have ‘disabled’ status compared to the effectiveDate (errorCode PY01)</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>Bic11Only</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="n"/>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n"/>
-      <c r="K6" s="12" t="n"/>
-      <c r="L6" s="12" t="n"/>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="12" t="n"/>
-      <c r="O6" s="12" t="n"/>
-      <c r="P6" s="12" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>initialSettBICValidityDate</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>settlementBIC</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>The Initial Parameter Validity Date set in the original command to be amended.
-**ValidationRule(s)** It must be present in routing repositories for the settlementBIC (errorCode DT01).</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="n"/>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="12" t="n"/>
-      <c r="L7" s="12" t="n"/>
-      <c r="M7" s="12" t="n"/>
-      <c r="N7" s="12" t="n"/>
-      <c r="O7" s="12" t="n"/>
-      <c r="P7" s="12" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>endSettBICValidityDate</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>settlementBIC</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>The End Parameter Validity Date set in the original command to be amended.
-**ValidationRule(s)** It must be present in routing repositories for the settlementBIC (errorCode DT01).</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="n"/>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="n"/>
-      <c r="K8" s="12" t="n"/>
-      <c r="L8" s="12" t="n"/>
-      <c r="M8" s="12" t="n"/>
-      <c r="N8" s="12" t="n"/>
-      <c r="O8" s="12" t="n"/>
-      <c r="P8" s="12" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="12" t="n"/>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n"/>
-      <c r="K9" s="12" t="n"/>
-      <c r="L9" s="12" t="n"/>
-      <c r="M9" s="12" t="n"/>
-      <c r="N9" s="12" t="n"/>
-      <c r="O9" s="12" t="n"/>
-      <c r="P9" s="12" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>settlBICName</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>The name of the Settlement BIC</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>ParticipantName</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="n"/>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n"/>
-      <c r="K10" s="12" t="n"/>
-      <c r="L10" s="12" t="n"/>
-      <c r="M10" s="12" t="n"/>
-      <c r="N10" s="12" t="n"/>
-      <c r="O10" s="12" t="n"/>
-      <c r="P10" s="12" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>automaticAdjustment</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>This parameter indicates if the Settlement BIC opts out of the automatic liquidity adjustments performed by the module at the EOL. In this case, thresholds are configured only to trigger alerts
-**ValidationRule(s)** Possible values
-true= automatic adjustment required
-false= automatic adjustment not required
-(errorCode SC01)</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="n"/>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n"/>
-      <c r="K11" s="12" t="n"/>
-      <c r="L11" s="12" t="n"/>
-      <c r="M11" s="12" t="n"/>
-      <c r="N11" s="12" t="n"/>
-      <c r="O11" s="12" t="n"/>
-      <c r="P11" s="12" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>eodFulDefund</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>This parameter indicates if the Settlement BIC opts for the CGS to perform an automatic full defunding of the Settlement BIC position on the last LAC of the business day in order to avoid remuneration of outstanding liquidity
-**ValidationRule(s)** Possible values
-true= EOD Full Defunding required
- false= EOD Full Defunding not required
-(errorCode SC01)</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="n"/>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n"/>
-      <c r="K12" s="12" t="n"/>
-      <c r="L12" s="12" t="n"/>
-      <c r="M12" s="12" t="n"/>
-      <c r="N12" s="12" t="n"/>
-      <c r="O12" s="12" t="n"/>
-      <c r="P12" s="12" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>lmrFileRequired</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>This parameter indicates whether the Settlement BIC must be configured to receive the LMR output file
-**ValidationRule(s)** Possible values
-true= LMR required
- false= LMR not required
-(errorCode SC01)</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="n"/>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J13" s="12" t="n"/>
-      <c r="K13" s="12" t="n"/>
-      <c r="L13" s="12" t="n"/>
-      <c r="M13" s="12" t="n"/>
-      <c r="N13" s="12" t="n"/>
-      <c r="O13" s="12" t="n"/>
-      <c r="P13" s="12" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>lnrFileRequired</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>This parameter indicates whether the Settlement BIC must be configured to receive the LNR output file
-**ValidationRule(s)** Possible values
-true= LNR required
- false= LNR not required
-(errorCode SC01)</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="n"/>
-      <c r="I14" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J14" s="12" t="n"/>
-      <c r="K14" s="12" t="n"/>
-      <c r="L14" s="12" t="n"/>
-      <c r="M14" s="12" t="n"/>
-      <c r="N14" s="12" t="n"/>
-      <c r="O14" s="12" t="n"/>
-      <c r="P14" s="12" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>dlrFileRequired</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>This parameter indicates whether the Settlement BIC must be configured to receive daily liquidity reconciliation report
-**ValidationRule(s)** Possible values
-true= daily liquidity reconciliation report required
-false= daily liquidity reconciliation report not required
-(errorCode SC01)</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F15" s="12" t="n"/>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>Boolean</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="n"/>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n"/>
-      <c r="K15" s="12" t="n"/>
-      <c r="L15" s="12" t="n"/>
-      <c r="M15" s="12" t="n"/>
-      <c r="N15" s="12" t="n"/>
-      <c r="O15" s="12" t="n"/>
-      <c r="P15" s="12" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>maxRcvgFileSize</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>settlementBICAmend</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>The maximum size of an output file generated and sent by the CGS to the Settlement BIC
-**ValidationRule(s)** The value must be in the range included between the default values set in the system for the Minimum file size and the Maximum file size.
-(errorCode XA15)</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="n"/>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="n"/>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n"/>
-      <c r="K16" s="12" t="n"/>
-      <c r="L16" s="12" t="n"/>
-      <c r="M16" s="12" t="n"/>
-      <c r="N16" s="12" t="n"/>
-      <c r="O16" s="12" t="n"/>
-      <c r="P16" s="12" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1 D3:D1048576">
@@ -1922,11 +1227,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="9" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
@@ -1938,6 +1243,53 @@
       <c r="B1" s="8" t="inlineStr">
         <is>
           <t>Body</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>dateTime: '2019-06-21T23:20:50.000001'
+settlementBIC:
+  settlementBICCode: IPSDID21XXX
+  initialSettBICValidityDate: '2019-06-21'
+  endSettBICValidityDate: '2024-11-08'
+settlementBICAmend:
+  settlBICName: ExampleBank01
+  automaticAdjustment: true
+  eodFulDefund: true
+  lmrFileRequired: true
+  lnrFileRequired: true
+  dlrFileRequired: true
+  maxRcvgFileSize: 0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Bad Request</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>settlementBIC:
+  settlementBICCode: IPSDID21XXX
+  initialSettBICValidityDate: '2019-06-21'
+  endSettBICValidityDate: '2024-11-08'
+settlementBICAmend:
+  settlBICName: ExampleBank01
+  automaticAdjustment: true
+  eodFulDefund: true
+  lmrFileRequired: true
+  lnrFileRequired: true
+  dlrFileRequired: true
+  maxRcvgFileSize: 0.0</t>
         </is>
       </c>
     </row>
@@ -1949,17 +1301,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFD3ECB9"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
     <col width="18" customWidth="1" style="3" min="2" max="2"/>
-    <col width="18" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
-    <col width="48" customWidth="1" style="3" min="4" max="4"/>
+    <col width="10" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
     <col width="18" customWidth="1" style="3" min="6" max="6"/>
     <col width="42" customWidth="1" style="3" min="7" max="7"/>
@@ -1971,7 +1323,7 @@
     <col width="10" customWidth="1" style="3" min="13" max="13"/>
     <col width="15" customWidth="1" style="3" min="14" max="14"/>
     <col width="10" customWidth="1" style="3" min="15" max="15"/>
-    <col width="10" customWidth="1" style="3" min="16" max="16"/>
+    <col width="9.140625" customWidth="1" style="3" min="16" max="16"/>
     <col width="9.140625" customWidth="1" style="3" min="17" max="16384"/>
   </cols>
   <sheetData>
@@ -2003,7 +1355,6 @@
       <c r="M1" s="6" t="n"/>
       <c r="N1" s="6" t="n"/>
       <c r="O1" s="6" t="n"/>
-      <c r="P1" s="12" t="n"/>
     </row>
     <row r="2" ht="43.15" customFormat="1" customHeight="1" s="4">
       <c r="A2" s="1" t="inlineStr">
@@ -2085,7 +1436,6 @@
           <t>Example</t>
         </is>
       </c>
-      <c r="P2" s="12" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -2123,99 +1473,6 @@
       <c r="M3" s="12" t="n"/>
       <c r="N3" s="12" t="n"/>
       <c r="O3" s="12" t="n"/>
-      <c r="P3" s="12" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>dateTime</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>The date and time of the API Response creation</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n"/>
-      <c r="K4" s="12" t="n"/>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>commandRef</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>The command reference</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>CommandReference</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n"/>
-      <c r="K5" s="12" t="n"/>
-      <c r="L5" s="12" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="12" t="n"/>
-      <c r="O5" s="12" t="n"/>
-      <c r="P5" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2226,15 +1483,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFD3ECB9"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
     <col width="12" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
     <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
@@ -2362,43 +1619,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>AmendChangeSettlementBICResponse</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -2408,17 +1628,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFFF9999"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="22" customWidth="1" style="3" min="2" max="2"/>
-    <col width="18" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
-    <col width="60" customWidth="1" style="3" min="4" max="4"/>
+    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="13" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
     <col width="18" customWidth="1" style="3" min="6" max="6"/>
     <col width="42" customWidth="1" style="3" min="7" max="7"/>
@@ -2430,7 +1650,7 @@
     <col width="10" customWidth="1" style="3" min="13" max="13"/>
     <col width="15" customWidth="1" style="3" min="14" max="14"/>
     <col width="10" customWidth="1" style="3" min="15" max="15"/>
-    <col width="10" customWidth="1" style="3" min="16" max="16"/>
+    <col width="9.140625" customWidth="1" style="3" min="16" max="16"/>
     <col width="9.140625" customWidth="1" style="3" min="17" max="16384"/>
   </cols>
   <sheetData>
@@ -2462,7 +1682,6 @@
       <c r="M1" s="6" t="n"/>
       <c r="N1" s="6" t="n"/>
       <c r="O1" s="6" t="n"/>
-      <c r="P1" s="12" t="n"/>
     </row>
     <row r="2" ht="43.15" customFormat="1" customHeight="1" s="4">
       <c r="A2" s="1" t="inlineStr">
@@ -2480,7 +1699,7 @@
           <t>Parent</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -2544,7 +1763,6 @@
           <t>Example</t>
         </is>
       </c>
-      <c r="P2" s="12" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -2558,7 +1776,7 @@
         </is>
       </c>
       <c r="C3" s="12" t="n"/>
-      <c r="D3" s="16" t="n"/>
+      <c r="D3" s="12" t="n"/>
       <c r="E3" s="12" t="inlineStr">
         <is>
           <t>schema</t>
@@ -2582,191 +1800,6 @@
       <c r="M3" s="12" t="n"/>
       <c r="N3" s="12" t="n"/>
       <c r="O3" s="12" t="n"/>
-      <c r="P3" s="12" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>dateTime</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>The date and time of the API Response creation</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n"/>
-      <c r="K4" s="12" t="n"/>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>errorCode</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>The relevant error code</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>ErrorCode</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n"/>
-      <c r="K5" s="12" t="n"/>
-      <c r="L5" s="12" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="12" t="n"/>
-      <c r="O5" s="12" t="n"/>
-      <c r="P5" s="12" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>errorCodeDescription</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>The description of the error</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>ErrorCodeDescription</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="n"/>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n"/>
-      <c r="K6" s="12" t="n"/>
-      <c r="L6" s="12" t="n"/>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="12" t="n"/>
-      <c r="O6" s="12" t="n"/>
-      <c r="P6" s="12" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>requestId</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>The automatically generated identification of the API request</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>RequestId</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="n"/>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="12" t="n"/>
-      <c r="L7" s="12" t="n"/>
-      <c r="M7" s="12" t="n"/>
-      <c r="N7" s="12" t="n"/>
-      <c r="O7" s="12" t="n"/>
-      <c r="P7" s="12" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2777,15 +1810,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFFF9999"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
     <col width="14" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
     <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
@@ -2913,43 +1946,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>ErrorResponse</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -2959,15 +1955,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFFF9999"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
     <col width="11" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
     <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
@@ -3095,43 +2091,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>ErrorResponse</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -3141,15 +2100,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Foglio16">
-    <tabColor theme="9" tint="0.5999938962981048"/>
+    <tabColor rgb="FFFF9999"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col width="10" customWidth="1" style="3" min="1" max="1"/>
-    <col width="18" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
     <col width="11" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
     <col width="13" customWidth="1" style="3" min="4" max="4"/>
     <col width="10" customWidth="1" style="3" min="5" max="5"/>
@@ -3277,43 +2236,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>schema</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>ErrorResponse</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="n"/>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n"/>
-      <c r="K3" s="12" t="n"/>
-      <c r="L3" s="12" t="n"/>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>